<commit_message>
moving around the UI
</commit_message>
<xml_diff>
--- a/Run_Log/1/StudentsSolution.xlsx
+++ b/Run_Log/1/StudentsSolution.xlsx
@@ -46,25 +46,25 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>04-12-2025 11:52:31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04-12-2025 11:54:24</x:t>
-  </x:si>
-  <x:si>
     <x:t>2</x:t>
   </x:si>
   <x:si>
+    <x:t>04-12-2025 12:43:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04-12-2025 12:45:05</x:t>
+  </x:si>
+  <x:si>
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
-    <x:t>4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04-12-2025 11:52:34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04-12-2025 11:53:29</x:t>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04-12-2025 12:43:21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04-12-2025 12:45:01</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
@@ -73,13 +73,10 @@
     <x:t>hoangbsthe186345</x:t>
   </x:si>
   <x:si>
-    <x:t>Failed</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04-12-2025 11:56:02</x:t>
+    <x:t>04-12-2025 12:43:22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04-12-2025 12:45:07</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -106,7 +103,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,11 +118,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF90EE90"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFB6C1"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -148,7 +140,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="4">
+  <x:cellStyleXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -158,11 +150,8 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -172,10 +161,6 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -522,18 +507,18 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="A3" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
         <x:v>13</x:v>
@@ -555,26 +540,26 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
-      <x:c r="A4" s="3" t="s">
+      <x:c r="A4" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="B4" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="C4" s="2" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="s">
+      <x:c r="D4" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="s">
+      <x:c r="G4" s="2" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="F4" s="3" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G4" s="3" t="s">
-        <x:v>21</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Proxy behavior still around
</commit_message>
<xml_diff>
--- a/Run_Log/1/StudentsSolution.xlsx
+++ b/Run_Log/1/StudentsSolution.xlsx
@@ -85,10 +85,13 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 02:55:36</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 02:57:09</x:t>
+    <x:t>1.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>08-12-2025 09:02:29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>08-12-2025 09:04:04</x:t>
   </x:si>
   <x:si>
     <x:t>7</x:t>
@@ -748,21 +751,21 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F7" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G7" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
         <x:v>7</x:v>
@@ -782,10 +785,10 @@
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
         <x:v>7</x:v>
@@ -805,10 +808,10 @@
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
         <x:v>7</x:v>
@@ -828,10 +831,10 @@
     </x:row>
     <x:row r="11" spans="1:7">
       <x:c r="A11" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
         <x:v>7</x:v>
@@ -851,10 +854,10 @@
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
         <x:v>7</x:v>
@@ -874,10 +877,10 @@
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="A13" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
         <x:v>7</x:v>
@@ -897,10 +900,10 @@
     </x:row>
     <x:row r="14" spans="1:7">
       <x:c r="A14" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>7</x:v>
@@ -920,10 +923,10 @@
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="A15" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
         <x:v>7</x:v>
@@ -943,10 +946,10 @@
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="A16" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
         <x:v>7</x:v>
@@ -966,10 +969,10 @@
     </x:row>
     <x:row r="17" spans="1:7">
       <x:c r="A17" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
         <x:v>7</x:v>
@@ -989,10 +992,10 @@
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="A18" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
         <x:v>7</x:v>
@@ -1012,10 +1015,10 @@
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="A19" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>7</x:v>
@@ -1035,10 +1038,10 @@
     </x:row>
     <x:row r="20" spans="1:7">
       <x:c r="A20" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>7</x:v>
@@ -1058,10 +1061,10 @@
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="A21" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
         <x:v>7</x:v>
@@ -1081,10 +1084,10 @@
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="A22" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
         <x:v>7</x:v>
@@ -1104,10 +1107,10 @@
     </x:row>
     <x:row r="23" spans="1:7">
       <x:c r="A23" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
         <x:v>7</x:v>
@@ -1127,10 +1130,10 @@
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="A24" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
         <x:v>7</x:v>
@@ -1150,10 +1153,10 @@
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="A25" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
         <x:v>7</x:v>
@@ -1173,10 +1176,10 @@
     </x:row>
     <x:row r="26" spans="1:7">
       <x:c r="A26" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
         <x:v>7</x:v>

</xml_diff>

<commit_message>
Network monitor unable to capture packages
</commit_message>
<xml_diff>
--- a/Run_Log/1/StudentsSolution.xlsx
+++ b/Run_Log/1/StudentsSolution.xlsx
@@ -49,10 +49,10 @@
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 11:57:13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 12:00:18</x:t>
+    <x:t>08-12-2025 12:09:48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>08-12-2025 12:12:39</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -61,7 +61,7 @@
     <x:t>anlpvhe187047</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 12:00:12</x:t>
+    <x:t>08-12-2025 12:12:40</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
@@ -70,7 +70,7 @@
     <x:t>cuongnvhe181200</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 12:00:15</x:t>
+    <x:t>08-12-2025 12:12:36</x:t>
   </x:si>
   <x:si>
     <x:t>4</x:t>
@@ -79,7 +79,7 @@
     <x:t>ducnthe180869</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 11:57:59</x:t>
+    <x:t>08-12-2025 12:10:52</x:t>
   </x:si>
   <x:si>
     <x:t>5</x:t>
@@ -88,10 +88,7 @@
     <x:t>dungdvhe181404</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 11:57:12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 12:00:11</x:t>
+    <x:t>08-12-2025 12:12:37</x:t>
   </x:si>
   <x:si>
     <x:t>6</x:t>
@@ -106,7 +103,7 @@
     <x:t>duongnthe186310</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 12:00:25</x:t>
+    <x:t>08-12-2025 12:12:26</x:t>
   </x:si>
   <x:si>
     <x:t>8</x:t>
@@ -121,13 +118,13 @@
     <x:t>duyldhe176352</x:t>
   </x:si>
   <x:si>
+    <x:t>08-12-2025 12:12:48</x:t>
+  </x:si>
+  <x:si>
     <x:t>10</x:t>
   </x:si>
   <x:si>
     <x:t>duynthe180374</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 12:00:10</x:t>
   </x:si>
   <x:si>
     <x:t>11</x:t>
@@ -749,18 +746,18 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F6" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="G6" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
       <x:c r="A7" s="2" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>27</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
         <x:v>7</x:v>
@@ -780,10 +777,10 @@
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="2" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
         <x:v>7</x:v>
@@ -798,15 +795,15 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G8" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="B9" s="2" t="s">
-        <x:v>32</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
         <x:v>7</x:v>
@@ -821,15 +818,15 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G9" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="s">
-        <x:v>34</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
         <x:v>7</x:v>
@@ -844,7 +841,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G10" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:7">
@@ -864,355 +861,355 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G11" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
       <x:c r="C12" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="A13" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
       <x:c r="C13" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G13" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:7">
       <x:c r="A14" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G14" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="A15" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
       <x:c r="C15" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G15" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="A16" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
       <x:c r="C16" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F16" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G16" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:7">
       <x:c r="A17" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
       <x:c r="C17" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G17" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="A18" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
       <x:c r="C18" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G18" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="A19" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G19" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:7">
       <x:c r="A20" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G20" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="A21" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
       <x:c r="C21" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F21" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G21" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="A22" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
       <x:c r="C22" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F22" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G22" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:7">
       <x:c r="A23" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
       <x:c r="C23" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F23" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G23" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="A24" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
       <x:c r="C24" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F24" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G24" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="A25" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>67</x:v>
-      </x:c>
       <x:c r="C25" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F25" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G25" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:7">
       <x:c r="A26" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
       <x:c r="C26" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F26" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G26" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
pushing sample run log
</commit_message>
<xml_diff>
--- a/Run_Log/1/StudentsSolution.xlsx
+++ b/Run_Log/1/StudentsSolution.xlsx
@@ -43,16 +43,16 @@
     <x:t>AnhDThe187386</x:t>
   </x:si>
   <x:si>
-    <x:t>Failed</x:t>
+    <x:t>Success</x:t>
   </x:si>
   <x:si>
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>08-12-2025 13:30:56</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 13:32:39</x:t>
+    <x:t>09-12-2025 15:59:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09-12-2025 16:01:02</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -89,9 +89,6 @@
   </x:si>
   <x:si>
     <x:t>dungtdhe186461</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08-12-2025 13:32:49</x:t>
   </x:si>
   <x:si>
     <x:t>7</x:t>
@@ -246,7 +243,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFB6C1"/>
+        <x:fgColor rgb="FF90EE90"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -738,34 +735,34 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
-      <x:c r="A7" s="2" t="s">
+      <x:c r="A7" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="s">
+      <x:c r="B7" s="0" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D7" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E7" s="2" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F7" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G7" s="2" t="s">
-        <x:v>25</x:v>
+      <x:c r="C7" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>27</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
         <x:v>7</x:v>
@@ -785,10 +782,10 @@
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
         <x:v>7</x:v>
@@ -808,10 +805,10 @@
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
         <x:v>7</x:v>
@@ -831,10 +828,10 @@
     </x:row>
     <x:row r="11" spans="1:7">
       <x:c r="A11" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>33</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
         <x:v>7</x:v>
@@ -854,10 +851,10 @@
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
         <x:v>7</x:v>
@@ -877,10 +874,10 @@
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="A13" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>37</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
         <x:v>7</x:v>
@@ -900,10 +897,10 @@
     </x:row>
     <x:row r="14" spans="1:7">
       <x:c r="A14" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>38</x:v>
-      </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>39</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>7</x:v>
@@ -923,10 +920,10 @@
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="A15" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
         <x:v>7</x:v>
@@ -946,10 +943,10 @@
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="A16" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
         <x:v>42</x:v>
-      </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>43</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
         <x:v>7</x:v>
@@ -969,10 +966,10 @@
     </x:row>
     <x:row r="17" spans="1:7">
       <x:c r="A17" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>44</x:v>
-      </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>45</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
         <x:v>7</x:v>
@@ -992,10 +989,10 @@
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="A18" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
         <x:v>46</x:v>
-      </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>47</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
         <x:v>7</x:v>
@@ -1015,10 +1012,10 @@
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="A19" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>49</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>7</x:v>
@@ -1038,10 +1035,10 @@
     </x:row>
     <x:row r="20" spans="1:7">
       <x:c r="A20" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>51</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>7</x:v>
@@ -1061,10 +1058,10 @@
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="A21" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
         <x:v>52</x:v>
-      </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>53</x:v>
       </x:c>
       <x:c r="C21" s="0" t="s">
         <x:v>7</x:v>
@@ -1084,10 +1081,10 @@
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="A22" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
         <x:v>54</x:v>
-      </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>55</x:v>
       </x:c>
       <x:c r="C22" s="0" t="s">
         <x:v>7</x:v>
@@ -1107,10 +1104,10 @@
     </x:row>
     <x:row r="23" spans="1:7">
       <x:c r="A23" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
         <x:v>7</x:v>
@@ -1130,10 +1127,10 @@
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="A24" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>59</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
         <x:v>7</x:v>
@@ -1153,10 +1150,10 @@
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="A25" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
         <x:v>7</x:v>
@@ -1176,10 +1173,10 @@
     </x:row>
     <x:row r="26" spans="1:7">
       <x:c r="A26" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>63</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
         <x:v>7</x:v>

</xml_diff>

<commit_message>
Revert "Merge pull request #137 from NguyenHuuCuongK18/copilot/fix-pcap-parsing-issue"
This reverts commit 55a741203f02bbce4d533a93410dd0cc44e0f64a, reversing
changes made to 67533b9d5ef27ad6d01fa48bd8182439aaed701a.
</commit_message>
<xml_diff>
--- a/Run_Log/1/StudentsSolution.xlsx
+++ b/Run_Log/1/StudentsSolution.xlsx
@@ -46,13 +46,13 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>1.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09-12-2025 16:37:12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09-12-2025 16:39:10</x:t>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09-12-2025 21:00:43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09-12-2025 21:02:41</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -64,9 +64,6 @@
     <x:t>Not Run</x:t>
   </x:si>
   <x:si>
-    <x:t>0</x:t>
-  </x:si>
-  <x:si>
     <x:t/>
   </x:si>
   <x:si>
@@ -94,7 +91,7 @@
     <x:t>dungtdhe186461</x:t>
   </x:si>
   <x:si>
-    <x:t>09-12-2025 16:41:18</x:t>
+    <x:t>09-12-2025 21:02:55</x:t>
   </x:si>
   <x:si>
     <x:t>7</x:t>
@@ -662,22 +659,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
       <x:c r="C4" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -685,22 +682,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="C5" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -708,22 +705,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="C6" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -731,21 +728,21 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
       <x:c r="A7" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>25</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
         <x:v>7</x:v>
@@ -754,22 +751,22 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G7" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
       <x:c r="C8" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -777,22 +774,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7">
       <x:c r="A9" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
       <x:c r="C9" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -800,22 +797,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G9" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
       <x:c r="A10" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
       <x:c r="C10" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -823,22 +820,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:7">
       <x:c r="A11" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
       <x:c r="C11" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -846,22 +843,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G11" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
       <x:c r="C12" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -869,22 +866,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="A13" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="C13" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -892,22 +889,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G13" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:7">
       <x:c r="A14" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -915,22 +912,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G14" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="A15" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
       <x:c r="C15" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -938,22 +935,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G15" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="A16" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B16" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="C16" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -961,22 +958,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F16" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G16" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:7">
       <x:c r="A17" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B17" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
       <x:c r="C17" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -984,22 +981,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G17" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="A18" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B18" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
       <x:c r="C18" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1007,22 +1004,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G18" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="A19" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B19" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1030,22 +1027,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G19" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:7">
       <x:c r="A20" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1053,22 +1050,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G20" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="A21" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B21" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="C21" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1076,22 +1073,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F21" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G21" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="A22" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B22" s="0" t="s">
-        <x:v>56</x:v>
-      </x:c>
       <x:c r="C22" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1099,22 +1096,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F22" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G22" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:7">
       <x:c r="A23" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B23" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
       <x:c r="C23" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1122,22 +1119,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F23" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G23" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="A24" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B24" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
       <x:c r="C24" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1145,22 +1142,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F24" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G24" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="A25" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
       <x:c r="C25" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1168,22 +1165,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F25" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G25" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:7">
       <x:c r="A26" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B26" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
       <x:c r="C26" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -1191,13 +1188,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F26" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G26" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>